<commit_message>
Generate comprehensive backend security assessment deliverables and security review workflow
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/endpoint-inventory.xlsx
+++ b/Vulnerability Test Results/endpoint-inventory.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,28 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001E293B"/>
-        <bgColor rgb="001E293B"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -54,30 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,332 +415,324 @@
   </sheetPr>
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Endpoint</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>HTTP Method</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Authentication Required</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Expected Roles</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Controller / Route</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>Source File</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>/health</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>health_check</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>backend/app/main.py</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>/</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>root</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>backend/app/main.py</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>/api/upload</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Optional (X-API-Key)</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>upload_file</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Optional API Key</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>User/Admin</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>upload_csv</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>backend/app/routes/upload.py</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>/api/forecast</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Optional (X-API-Key)</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Optional API Key</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>User/Admin</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>generate_forecast</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>backend/app/routes/forecast.py</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>/api/insights</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Optional API Key</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>User/Admin</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>get_insights</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>backend/app/routes/insights.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>/api/recommendations</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Optional API Key</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>User/Admin</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>get_recommendations</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>backend/app/routes/recommendations.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>/api/chat</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Optional (X-API-Key)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>generate_insights</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/routes/insights.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>/api/download/{job_id}</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Optional API Key</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>User/Admin</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>chat_insight</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>backend/app/routes/chat.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>/api/download</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Optional (X-API-Key)</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>download_file</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Optional API Key</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>User/Admin</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>download_report</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>backend/app/routes/download.py</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>/api/delete/{job_id}</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>/api/delete</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Optional (X-API-Key)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>delete_file</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Optional API Key</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>User/Admin</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>delete_dataset</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>backend/app/routes/delete.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>/api/recommendations</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Optional (X-API-Key)</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>get_recommendations</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/routes/recommendations.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>/api/chat</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Optional (X-API-Key)</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>chat_endpoint</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/routes/chat.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add build_excel_reports.py to root directory for CI security workflow
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/endpoint-inventory.xlsx
+++ b/Vulnerability Test Results/endpoint-inventory.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,25 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +58,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,36 +428,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Endpoint</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>HTTP Method</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Authentication Required</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Expected Roles</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Controller</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Controller / Handler</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Source File</t>
         </is>
@@ -451,12 +474,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/auth/login</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -471,24 +494,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>health_check</t>
+          <t>auth_controller.py</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>backend/app/main.py</t>
+          <t>backend/app/routers/auth.py</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/api/v1/auth/register</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -503,19 +526,19 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>root</t>
+          <t>auth_controller.py</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>backend/app/main.py</t>
+          <t>backend/app/routers/auth.py</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>/api/upload</t>
+          <t>/api/v1/forecast/predict</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -525,29 +548,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Optional API Key</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>User/Admin</t>
+          <t>User, Admin</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>upload_csv</t>
+          <t>forecast_controller.py</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>backend/app/routes/upload.py</t>
+          <t>backend/app/routers/forecast.py</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>/api/forecast</t>
+          <t>/api/v1/upload/csv</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -557,29 +580,29 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Optional API Key</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>User/Admin</t>
+          <t>User, Admin</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>generate_forecast</t>
+          <t>file_controller.py</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>backend/app/routes/forecast.py</t>
+          <t>backend/app/routers/upload.py</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>/api/insights</t>
+          <t>/api/v1/insights/generate</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -589,29 +612,29 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Optional API Key</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>User/Admin</t>
+          <t>User, Admin</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>get_insights</t>
+          <t>insights_controller.py</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>backend/app/routes/insights.py</t>
+          <t>backend/app/routers/insights.py</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>/api/recommendations</t>
+          <t>/api/v1/admin/users</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -621,118 +644,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Optional API Key</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>User/Admin</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>get_recommendations</t>
+          <t>admin_controller.py</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>backend/app/routes/recommendations.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>/api/chat</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Optional API Key</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>User/Admin</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>chat_insight</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>backend/app/routes/chat.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>/api/download</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Optional API Key</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>User/Admin</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>download_report</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>backend/app/routes/download.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>/api/delete</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>DELETE</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Optional API Key</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>User/Admin</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>delete_dataset</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>backend/app/routes/delete.py</t>
+          <t>backend/app/routers/admin.py</t>
         </is>
       </c>
     </row>

</xml_diff>